<commit_message>
fix source file upload
</commit_message>
<xml_diff>
--- a/source_data_replication.xlsx
+++ b/source_data_replication.xlsx
@@ -66,7 +66,7 @@
     <t xml:space="preserve">change</t>
   </si>
   <si>
-    <t xml:space="preserve">REPLICATION</t>
+    <t xml:space="preserve">sample</t>
   </si>
   <si>
     <t xml:space="preserve">scale(PGSS_AD_Jansen)</t>
@@ -81,7 +81,7 @@
     <t xml:space="preserve">ageRelChange</t>
   </si>
   <si>
-    <t xml:space="preserve">REPLICATION_RESULTS</t>
+    <t xml:space="preserve">REPLICATION</t>
   </si>
   <si>
     <t xml:space="preserve">scale(PGSS_AD)</t>
@@ -529,7 +529,7 @@
     <col min="14" max="14" width="11.71" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="11.71" hidden="0" customWidth="1"/>
     <col min="16" max="16" width="12.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="19.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6548,7 +6548,7 @@
     <col min="14" max="14" width="11.71" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="11.71" hidden="0" customWidth="1"/>
     <col min="16" max="16" width="12.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="19.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11623,7 +11623,7 @@
     <col min="14" max="14" width="11.71" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="11.71" hidden="0" customWidth="1"/>
     <col min="16" max="16" width="12.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="19.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -17642,7 +17642,7 @@
     <col min="14" max="14" width="8.71" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="8.71" hidden="0" customWidth="1"/>
     <col min="16" max="16" width="12.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="19.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21869,7 +21869,7 @@
     <col min="14" max="14" width="8.71" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="11.71" hidden="0" customWidth="1"/>
     <col min="16" max="16" width="12.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="3.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21921,7 +21921,9 @@
       <c r="P1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="Q1" s="1"/>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -21972,6 +21974,9 @@
       <c r="P2" t="s">
         <v>42</v>
       </c>
+      <c r="Q2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -22022,6 +22027,9 @@
       <c r="P3" t="s">
         <v>42</v>
       </c>
+      <c r="Q3" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -22072,6 +22080,9 @@
       <c r="P4" t="s">
         <v>42</v>
       </c>
+      <c r="Q4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -22122,6 +22133,9 @@
       <c r="P5" t="s">
         <v>42</v>
       </c>
+      <c r="Q5" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -22172,6 +22186,9 @@
       <c r="P6" t="s">
         <v>42</v>
       </c>
+      <c r="Q6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -22222,6 +22239,9 @@
       <c r="P7" t="s">
         <v>42</v>
       </c>
+      <c r="Q7" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -22272,6 +22292,9 @@
       <c r="P8" t="s">
         <v>42</v>
       </c>
+      <c r="Q8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -22322,6 +22345,9 @@
       <c r="P9" t="s">
         <v>42</v>
       </c>
+      <c r="Q9" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -22372,6 +22398,9 @@
       <c r="P10" t="s">
         <v>42</v>
       </c>
+      <c r="Q10" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -22422,6 +22451,9 @@
       <c r="P11" t="s">
         <v>42</v>
       </c>
+      <c r="Q11" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -22472,6 +22504,9 @@
       <c r="P12" t="s">
         <v>42</v>
       </c>
+      <c r="Q12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -22522,6 +22557,9 @@
       <c r="P13" t="s">
         <v>42</v>
       </c>
+      <c r="Q13" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -22572,6 +22610,9 @@
       <c r="P14" t="s">
         <v>42</v>
       </c>
+      <c r="Q14" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -22622,6 +22663,9 @@
       <c r="P15" t="s">
         <v>42</v>
       </c>
+      <c r="Q15" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -22672,6 +22716,9 @@
       <c r="P16" t="s">
         <v>42</v>
       </c>
+      <c r="Q16" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -22722,6 +22769,9 @@
       <c r="P17" t="s">
         <v>42</v>
       </c>
+      <c r="Q17" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -22772,6 +22822,9 @@
       <c r="P18" t="s">
         <v>42</v>
       </c>
+      <c r="Q18" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -22822,6 +22875,9 @@
       <c r="P19" t="s">
         <v>42</v>
       </c>
+      <c r="Q19" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -22872,6 +22928,9 @@
       <c r="P20" t="s">
         <v>42</v>
       </c>
+      <c r="Q20" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -22922,6 +22981,9 @@
       <c r="P21" t="s">
         <v>42</v>
       </c>
+      <c r="Q21" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -22971,6 +23033,9 @@
       </c>
       <c r="P22" t="s">
         <v>42</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="23">
@@ -23022,6 +23087,9 @@
       <c r="P23" t="s">
         <v>42</v>
       </c>
+      <c r="Q23" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -23072,6 +23140,9 @@
       <c r="P24" t="s">
         <v>42</v>
       </c>
+      <c r="Q24" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -23122,6 +23193,9 @@
       <c r="P25" t="s">
         <v>42</v>
       </c>
+      <c r="Q25" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -23172,6 +23246,9 @@
       <c r="P26" t="s">
         <v>42</v>
       </c>
+      <c r="Q26" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -23222,6 +23299,9 @@
       <c r="P27" t="s">
         <v>42</v>
       </c>
+      <c r="Q27" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -23272,6 +23352,9 @@
       <c r="P28" t="s">
         <v>42</v>
       </c>
+      <c r="Q28" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -23321,6 +23404,9 @@
       </c>
       <c r="P29" t="s">
         <v>42</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>